<commit_message>
Documents à télécharger alignés sur le site (domaine, adresse, architecture, tailles)
Data Book : 40 liens enertchad-delta.vercel.app → enertchad.com (ancres corrigées), adresse du siège, « 8 pôles » → 3 pôles de cœur + pétrochimie + 4 capacités, « société créée » → « constitution engagée », date d’extraction 9 octobre 2026. Dossier investisseur : adresse du siège. Fiche investisseur : ancien domaine remplacé. Fiche Intermédiaire et Point d’étape régénérés depuis docs-sources. Tailles affichées des documents corrigées (ex. brochure 211 → 606 Ko, fiche arabe 316 → 345 Ko).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01924b9tNJjnMM63pEUTgBf9
</commit_message>
<xml_diff>
--- a/Data_Book_EnerTchad.xlsx
+++ b/Data_Book_EnerTchad.xlsx
@@ -528,7 +528,7 @@
     <x:row r="11" s="15" customFormat="1" ht="15" customHeight="1">
       <x:c r="A11" s="18" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Extraction : 28 aout 2026, depuis le site officiel https://enertchad-delta.vercel.app</x:t>
+          <x:t xml:space="preserve">Extraction : 9 octobre 2026, depuis le site officiel https://enertchad.com</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -615,7 +615,7 @@
       </x:c>
       <x:c r="D2" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/societe</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/societe</x:t>
         </x:is>
       </x:c>
       <x:c r="E2" s="20" t="inlineStr">
@@ -642,7 +642,7 @@
       </x:c>
       <x:c r="D3" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/societe</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/societe</x:t>
         </x:is>
       </x:c>
       <x:c r="E3" s="21" t="inlineStr">
@@ -669,7 +669,7 @@
       </x:c>
       <x:c r="D4" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/societe</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/societe</x:t>
         </x:is>
       </x:c>
       <x:c r="E4" s="20" t="inlineStr">
@@ -696,7 +696,7 @@
       </x:c>
       <x:c r="D5" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/societe</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/societe</x:t>
         </x:is>
       </x:c>
       <x:c r="E5" s="21" t="inlineStr">
@@ -713,7 +713,7 @@
       </x:c>
       <x:c r="B6" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Block D, 2e étage, bureau 23, Quartier Sabangali, Cité du 1er décembre, N'Djamena, Tchad</x:t>
+          <x:t xml:space="preserve">Radisson Blu, bureau 23, Quartier Sabangali, Cité du 1er Décembre, BP 6060, N'Djamena, Tchad</x:t>
         </x:is>
       </x:c>
       <x:c r="C6" s="20" t="inlineStr">
@@ -723,7 +723,7 @@
       </x:c>
       <x:c r="D6" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/contact</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/contact</x:t>
         </x:is>
       </x:c>
       <x:c r="E6" s="20" t="inlineStr">
@@ -750,7 +750,7 @@
       </x:c>
       <x:c r="D7" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/societe</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/societe</x:t>
         </x:is>
       </x:c>
       <x:c r="E7" s="21" t="inlineStr">
@@ -775,7 +775,7 @@
       </x:c>
       <x:c r="D8" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/</x:t>
         </x:is>
       </x:c>
       <x:c r="E8" s="20" t="inlineStr">
@@ -792,7 +792,7 @@
       </x:c>
       <x:c r="B9" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Societe unique (pas un groupe) — 8 poles d'activite internes</x:t>
+          <x:t xml:space="preserve">Societe unique (pas un groupe) — 3 poles de coeur, petrochimie, 4 capacites integrees</x:t>
         </x:is>
       </x:c>
       <x:c r="C9" s="21" t="inlineStr">
@@ -802,7 +802,7 @@
       </x:c>
       <x:c r="D9" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/societe#poles</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/societe#organisation</x:t>
         </x:is>
       </x:c>
       <x:c r="E9" s="21" t="inlineStr">
@@ -829,7 +829,7 @@
       </x:c>
       <x:c r="D10" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/societe#poles</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/societe#organisation</x:t>
         </x:is>
       </x:c>
       <x:c r="E10" s="20" t="inlineStr">
@@ -856,7 +856,7 @@
       </x:c>
       <x:c r="D11" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/societe#poles</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/societe#organisation</x:t>
         </x:is>
       </x:c>
       <x:c r="E11" s="21" t="inlineStr">
@@ -883,7 +883,7 @@
       </x:c>
       <x:c r="D12" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/</x:t>
         </x:is>
       </x:c>
       <x:c r="E12" s="20" t="inlineStr">
@@ -910,7 +910,7 @@
       </x:c>
       <x:c r="D13" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/investisseurs</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/investisseurs</x:t>
         </x:is>
       </x:c>
       <x:c r="E13" s="21" t="inlineStr">
@@ -986,12 +986,12 @@
       </x:c>
       <x:c r="D2" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">fait — 100 % tchadien, societe creee</x:t>
+          <x:t xml:space="preserve">en cours — 100 % tchadien, constitution engagee</x:t>
         </x:is>
       </x:c>
       <x:c r="E2" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/investisseurs#jalons</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/investisseurs#jalons</x:t>
         </x:is>
       </x:c>
       <x:c r="F2" s="20" t="inlineStr">
@@ -1023,7 +1023,7 @@
       </x:c>
       <x:c r="E3" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/investisseurs#jalons</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/investisseurs#jalons</x:t>
         </x:is>
       </x:c>
       <x:c r="F3" s="21" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </x:c>
       <x:c r="E4" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/investisseurs#jalons</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/investisseurs#jalons</x:t>
         </x:is>
       </x:c>
       <x:c r="F4" s="20" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </x:c>
       <x:c r="E5" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/investisseurs#jalons</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/investisseurs#jalons</x:t>
         </x:is>
       </x:c>
       <x:c r="F5" s="21" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </x:c>
       <x:c r="E6" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/investisseurs#jalons</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/investisseurs#jalons</x:t>
         </x:is>
       </x:c>
       <x:c r="F6" s="20" t="inlineStr">
@@ -1151,7 +1151,7 @@
       </x:c>
       <x:c r="E7" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/investisseurs#agenda</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/investisseurs#agenda</x:t>
         </x:is>
       </x:c>
       <x:c r="F7" s="21" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </x:c>
       <x:c r="E8" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/investisseurs#agenda</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/investisseurs#agenda</x:t>
         </x:is>
       </x:c>
       <x:c r="F8" s="20" t="inlineStr">
@@ -1215,7 +1215,7 @@
       </x:c>
       <x:c r="E9" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/investisseurs#agenda</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/investisseurs#agenda</x:t>
         </x:is>
       </x:c>
       <x:c r="F9" s="21" t="inlineStr">
@@ -1247,7 +1247,7 @@
       </x:c>
       <x:c r="E10" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/agenda-investisseur.ics</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/agenda-investisseur.ics</x:t>
         </x:is>
       </x:c>
       <x:c r="F10" s="20" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </x:c>
       <x:c r="E2" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/cibles-2030</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/cibles-2030</x:t>
         </x:is>
       </x:c>
       <x:c r="F2" s="20" t="inlineStr">
@@ -1360,7 +1360,7 @@
       </x:c>
       <x:c r="E3" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/cibles-2030</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/cibles-2030</x:t>
         </x:is>
       </x:c>
       <x:c r="F3" s="21" t="inlineStr">
@@ -1392,7 +1392,7 @@
       </x:c>
       <x:c r="E4" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/cibles-2030</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/cibles-2030</x:t>
         </x:is>
       </x:c>
       <x:c r="F4" s="20" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </x:c>
       <x:c r="E5" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/cibles-2030</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/cibles-2030</x:t>
         </x:is>
       </x:c>
       <x:c r="F5" s="21" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </x:c>
       <x:c r="E6" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/cibles-2030</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/cibles-2030</x:t>
         </x:is>
       </x:c>
       <x:c r="F6" s="20" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </x:c>
       <x:c r="E7" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/cibles-2030</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/cibles-2030</x:t>
         </x:is>
       </x:c>
       <x:c r="F7" s="21" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </x:c>
       <x:c r="E8" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/aval/raffinage</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/aval/raffinage</x:t>
         </x:is>
       </x:c>
       <x:c r="F8" s="20" t="inlineStr">
@@ -1552,7 +1552,7 @@
       </x:c>
       <x:c r="E9" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/cibles-2030</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/cibles-2030</x:t>
         </x:is>
       </x:c>
       <x:c r="F9" s="21" t="inlineStr">
@@ -1584,7 +1584,7 @@
       </x:c>
       <x:c r="E10" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/cibles-2030</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/cibles-2030</x:t>
         </x:is>
       </x:c>
       <x:c r="F10" s="20" t="inlineStr">
@@ -1616,7 +1616,7 @@
       </x:c>
       <x:c r="E11" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/cibles-2030</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/cibles-2030</x:t>
         </x:is>
       </x:c>
       <x:c r="F11" s="21" t="inlineStr">
@@ -1761,7 +1761,7 @@
     <x:row r="10" s="15" customFormat="1" ht="15" customHeight="1">
       <x:c r="A10" s="27" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Allocation cible et indicative des fonds propres recherches — ajustable au rythme des levees ; arretee au closing de chaque tranche. Source : https://enertchad-delta.vercel.app/investisseurs#affectation</x:t>
+          <x:t xml:space="preserve">Allocation cible et indicative des fonds propres recherches — ajustable au rythme des levees ; arretee au closing de chaque tranche. Source : https://enertchad.com/investisseurs#affectation</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1837,7 +1837,7 @@
       </x:c>
       <x:c r="E2" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/enerconseils/atlas#donnees-secteur</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/atlas/cadre-sectoriel</x:t>
         </x:is>
       </x:c>
       <x:c r="F2" s="20" t="inlineStr">
@@ -1869,7 +1869,7 @@
       </x:c>
       <x:c r="E3" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/enerconseils/atlas#donnees-secteur</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/atlas/cadre-sectoriel</x:t>
         </x:is>
       </x:c>
       <x:c r="F3" s="21" t="inlineStr">
@@ -1901,7 +1901,7 @@
       </x:c>
       <x:c r="E4" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/intermediaire/logistique</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/intermediaire/logistique</x:t>
         </x:is>
       </x:c>
       <x:c r="F4" s="20" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </x:c>
       <x:c r="E5" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/investisseurs</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/investisseurs</x:t>
         </x:is>
       </x:c>
       <x:c r="F5" s="21" t="inlineStr">
@@ -1965,7 +1965,7 @@
       </x:c>
       <x:c r="E6" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/investisseurs</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/investisseurs</x:t>
         </x:is>
       </x:c>
       <x:c r="F6" s="20" t="inlineStr">
@@ -1997,7 +1997,7 @@
       </x:c>
       <x:c r="E7" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/investisseurs</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/investisseurs</x:t>
         </x:is>
       </x:c>
       <x:c r="F7" s="21" t="inlineStr">
@@ -2029,7 +2029,7 @@
       </x:c>
       <x:c r="E8" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://enertchad-delta.vercel.app/investisseurs</x:t>
+          <x:t xml:space="preserve">https://enertchad.com/investisseurs</x:t>
         </x:is>
       </x:c>
       <x:c r="F8" s="20" t="inlineStr">

</xml_diff>

<commit_message>
Dates : plan du site, étagère investisseur et agenda des documents à jour
sitemap.xml : lastmod recalculé depuis l’historique Git (217 URL au 9 octobre 2026 ; 197 restaient au 29 septembre). /investisseurs (FR/EN) : dates des quatre documents mises à octobre 2026, point d’étape « mis à jour en octobre ». Data Book et Point d’étape : agenda aligné sur le site (mémorandum et webinaire T4 2026, data room T1 2027).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01924b9tNJjnMM63pEUTgBf9
</commit_message>
<xml_diff>
--- a/Data_Book_EnerTchad.xlsx
+++ b/Data_Book_EnerTchad.xlsx
@@ -1136,7 +1136,7 @@
       </x:c>
       <x:c r="B7" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">T3 2026</x:t>
+          <x:t xml:space="preserve">T4 2026</x:t>
         </x:is>
       </x:c>
       <x:c r="C7" s="21" t="inlineStr">
@@ -1168,7 +1168,7 @@
       </x:c>
       <x:c r="B8" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">T3 2026</x:t>
+          <x:t xml:space="preserve">T4 2026</x:t>
         </x:is>
       </x:c>
       <x:c r="C8" s="20" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </x:c>
       <x:c r="B9" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">T4 2026</x:t>
+          <x:t xml:space="preserve">T1 2027</x:t>
         </x:is>
       </x:c>
       <x:c r="C9" s="21" t="inlineStr">
@@ -1220,7 +1220,7 @@
       </x:c>
       <x:c r="F9" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">2026</x:t>
+          <x:t xml:space="preserve">2027</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Amont lot 3 (2) : gouvernance, investisseurs, glossaire, journaux, mentions et Data book alignés
Décisions du DG du 20 octobre 2026 : méthane (Zero Routine Flaring, OGMP 2.0) et HSE (IOGP) sur gouvernance ; premier baril expliqué (6-12 mois anticipé, ≤ 24 mois complet) ; mentions de dépôt de marque retirées (aucun dépôt) ; Data book : 2P retiré, capital « Fait », oléoduc ~55 % (ITIE 2023, COTCO).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01924b9tNJjnMM63pEUTgBf9
</commit_message>
<xml_diff>
--- a/Data_Book_EnerTchad.xlsx
+++ b/Data_Book_EnerTchad.xlsx
@@ -1004,7 +1004,7 @@
       </c>
       <c r="D2" s="20" t="inlineStr">
         <is>
-          <t>en cours — 100 % tchadien, constitution engagee</t>
+          <t>Fait — capital fondateur de 100 M FCFA réuni</t>
         </is>
       </c>
       <c r="E2" s="20" t="inlineStr">
@@ -2079,27 +2079,27 @@
       </c>
       <c r="B9" s="20" t="inlineStr">
         <is>
-          <t>~2,8</t>
+          <t>2P non publiées</t>
         </is>
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
-          <t>Gbep</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D9" s="20" t="inlineStr">
         <is>
-          <t>estimation a confirmer — source en cours de verification</t>
+          <t>contexte — 2P non publiées ; seules les réserves prouvées sont sourcées : 1,5 Gb en 2018 (trade.gov)</t>
         </is>
       </c>
       <c r="E9" s="20" t="inlineStr">
         <is>
-          <t>https://enertchad.com/investisseurs#marche</t>
+          <t>https://enertchad.com/amont/reserves</t>
         </is>
       </c>
       <c r="F9" s="20" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
@@ -2111,7 +2111,7 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>~40</t>
+          <t>~55</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
@@ -2121,7 +2121,7 @@
       </c>
       <c r="D10" s="20" t="inlineStr">
         <is>
-          <t>estimation a confirmer — source en cours de verification</t>
+          <t>contexte — ~45 % de capacité disponible (ITIE 2023, COTCO)</t>
         </is>
       </c>
       <c r="E10" s="20" t="inlineStr">
@@ -2131,7 +2131,7 @@
       </c>
       <c r="F10" s="20" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
@@ -2185,7 +2185,7 @@
       </c>
       <c r="D12" s="20" t="inlineStr">
         <is>
-          <t>estimation a confirmer — source en cours de verification — contre 3 a 5 ans en developpement conventionnel</t>
+          <t>cible — 6 à 12 mois en production anticipée (unité de traitement provisoire), ≤ 24 mois jusqu’au développement complet, sur un champ déjà découvert et sous réserve d’accès — contre 3 à 5 ans en développement conventionnel</t>
         </is>
       </c>
       <c r="E12" s="20" t="inlineStr">

</xml_diff>

<commit_message>
OVH: reviewed corporate readiness export from 83f008474c8fdb2a52398d70b227dc27b8ad2d0c
</commit_message>
<xml_diff>
--- a/Data_Book_EnerTchad.xlsx
+++ b/Data_Book_EnerTchad.xlsx
@@ -1004,7 +1004,7 @@
       </c>
       <c r="D2" s="20" t="inlineStr">
         <is>
-          <t>en cours — 100 % tchadien, constitution engagee</t>
+          <t>Fait — capital fondateur de 100 M FCFA réuni</t>
         </is>
       </c>
       <c r="E2" s="20" t="inlineStr">
@@ -2079,27 +2079,27 @@
       </c>
       <c r="B9" s="20" t="inlineStr">
         <is>
-          <t>~2,8</t>
+          <t>2P non publiées</t>
         </is>
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
-          <t>Gbep</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D9" s="20" t="inlineStr">
         <is>
-          <t>estimation a confirmer — source en cours de verification</t>
+          <t>contexte — 2P non publiées ; seules les réserves prouvées sont sourcées : 1,5 Gb en 2018 (trade.gov)</t>
         </is>
       </c>
       <c r="E9" s="20" t="inlineStr">
         <is>
-          <t>https://enertchad.com/investisseurs#marche</t>
+          <t>https://enertchad.com/amont/reserves</t>
         </is>
       </c>
       <c r="F9" s="20" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
@@ -2111,7 +2111,7 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>~40</t>
+          <t>~55</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
@@ -2121,7 +2121,7 @@
       </c>
       <c r="D10" s="20" t="inlineStr">
         <is>
-          <t>estimation a confirmer — source en cours de verification</t>
+          <t>contexte — ~45 % de capacité disponible (ITIE 2023, COTCO)</t>
         </is>
       </c>
       <c r="E10" s="20" t="inlineStr">
@@ -2131,7 +2131,7 @@
       </c>
       <c r="F10" s="20" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
@@ -2185,7 +2185,7 @@
       </c>
       <c r="D12" s="20" t="inlineStr">
         <is>
-          <t>estimation a confirmer — source en cours de verification — contre 3 a 5 ans en developpement conventionnel</t>
+          <t>cible — 6 à 12 mois en production anticipée (unité de traitement provisoire), ≤ 24 mois jusqu’au développement complet, sur un champ déjà découvert et sous réserve d’accès — contre 3 à 5 ans en développement conventionnel</t>
         </is>
       </c>
       <c r="E12" s="20" t="inlineStr">

</xml_diff>

<commit_message>
Lot 21 (13/13) : journal, communiqués EN, flux RSS (note CP-004), Data Book (cible nationale 250 kb/j)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01924b9tNJjnMM63pEUTgBf9
</commit_message>
<xml_diff>
--- a/Data_Book_EnerTchad.xlsx
+++ b/Data_Book_EnerTchad.xlsx
@@ -532,14 +532,14 @@
     <row r="11" ht="15" customHeight="1" s="15">
       <c r="A11" s="18" t="inlineStr">
         <is>
-          <t>Extraction : 18 octobre 2026, depuis le site officiel https://enertchad.com</t>
+          <t>Extraction : 18 octobre 2026, depuis le site officiel https://enertchad.com ; mise à jour : 23 octobre 2026</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="15">
       <c r="A12" s="18" t="inlineStr">
         <is>
-          <t>Contact investisseurs : contact@enertchad.com · +235 30 16 26 26 · Partenaire investissement : GCIC</t>
+          <t>Contact investisseurs : contact@enertchad.com · +235 30 16 26 26 · Conseil pressenti : GCIC</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="15">
+    <row r="9" ht="23.25" customHeight="1" s="15">
       <c r="A9" s="21" t="inlineStr">
         <is>
           <t>Organisation</t>
@@ -805,7 +805,7 @@
       </c>
       <c r="B9" s="21" t="inlineStr">
         <is>
-          <t>Societe unique (pas un groupe) — 3 poles de coeur, petrochimie, 4 capacites integrees</t>
+          <t>Société unique (pas un groupe) — 4 segments industriels + 4 capacités intégrées</t>
         </is>
       </c>
       <c r="C9" s="21" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="10" ht="15" customHeight="1" s="15">
       <c r="A10" s="20" t="inlineStr">
         <is>
-          <t>Poles chaine (4)</t>
+          <t>Segments industriels (4)</t>
         </is>
       </c>
       <c r="B10" s="20" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="11" ht="15" customHeight="1" s="15">
       <c r="A11" s="21" t="inlineStr">
         <is>
-          <t>Poles supports (4)</t>
+          <t>Capacités intégrées (4)</t>
         </is>
       </c>
       <c r="B11" s="21" t="inlineStr">
@@ -908,17 +908,17 @@
     <row r="13" ht="15" customHeight="1" s="15">
       <c r="A13" s="21" t="inlineStr">
         <is>
-          <t>Partenaire investissement</t>
+          <t>Conseil pressenti (levées)</t>
         </is>
       </c>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>GCIC</t>
+          <t>GCIC (Guess Consulting &amp; Investment Capital)</t>
         </is>
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
-          <t>fait</t>
+          <t>cible</t>
         </is>
       </c>
       <c r="D13" s="21" t="inlineStr">
@@ -1050,7 +1050,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="15">
+    <row r="4" ht="23.25" customHeight="1" s="15">
       <c r="A4" s="20" t="inlineStr">
         <is>
           <t>1re levee visee</t>
@@ -1068,7 +1068,7 @@
       </c>
       <c r="D4" s="20" t="inlineStr">
         <is>
-          <t>cible — court terme, tours d'amorcage avec GCIC ; montant non publie</t>
+          <t>cible — court terme, tours d'amorçage (GCIC, conseil pressenti) ; montant non publié</t>
         </is>
       </c>
       <c r="E4" s="20" t="inlineStr">
@@ -1114,10 +1114,10 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="15">
+    <row r="6" ht="23.25" customHeight="1" s="15">
       <c r="A6" s="20" t="inlineStr">
         <is>
-          <t>Capital vise a cinq ans</t>
+          <t>Capital visé</t>
         </is>
       </c>
       <c r="B6" s="20" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>cible — a cinq ans, levees successives ; montant non publie</t>
+          <t>cible — levées successives par paliers ; montant non publié</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
@@ -1210,10 +1210,10 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="15">
+    <row r="9" ht="23.25" customHeight="1" s="15">
       <c r="A9" s="21" t="inlineStr">
         <is>
-          <t>Data room &amp; rencontres (GCIC)</t>
+          <t>Data room &amp; rencontres (GCIC, conseil pressenti)</t>
         </is>
       </c>
       <c r="B9" s="21" t="inlineStr">
@@ -1328,10 +1328,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="15">
+    <row r="2" ht="23.25" customHeight="1" s="15">
       <c r="A2" s="20" t="inlineStr">
         <is>
-          <t>Production visee</t>
+          <t>Production nationale visée par le plan 2025-2030</t>
         </is>
       </c>
       <c r="B2" s="20" t="inlineStr">
@@ -1346,7 +1346,7 @@
       </c>
       <c r="D2" s="20" t="inlineStr">
         <is>
-          <t>cible 2030</t>
+          <t>contexte — EnerTchad y contribue ; pas une cible propre</t>
         </is>
       </c>
       <c r="E2" s="20" t="inlineStr">
@@ -1360,20 +1360,20 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" s="15">
+    <row r="3" ht="23.25" customHeight="1" s="15">
       <c r="A3" s="21" t="inlineStr">
         <is>
-          <t>Poles d'activite</t>
+          <t>Segments industriels + capacités intégrées</t>
         </is>
       </c>
       <c r="B3" s="21" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4 + 4</t>
         </is>
       </c>
       <c r="C3" s="21" t="inlineStr">
         <is>
-          <t>poles</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D3" s="21" t="inlineStr">
@@ -1424,7 +1424,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="15">
+    <row r="5" ht="23.25" customHeight="1" s="15">
       <c r="A5" s="21" t="inlineStr">
         <is>
           <t>Capital cible</t>
@@ -1442,7 +1442,7 @@
       </c>
       <c r="D5" s="21" t="inlineStr">
         <is>
-          <t>cible a cinq ans — levees successives, montant non publie</t>
+          <t>cible — levées successives par paliers, montant non publié</t>
         </is>
       </c>
       <c r="E5" s="21" t="inlineStr">
@@ -1452,7 +1452,7 @@
       </c>
       <c r="F5" s="21" t="inlineStr">
         <is>
-          <t>2031</t>
+          <t>par paliers</t>
         </is>
       </c>
     </row>
@@ -1488,7 +1488,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="15">
+    <row r="7" ht="23.25" customHeight="1" s="15">
       <c r="A7" s="21" t="inlineStr">
         <is>
           <t>Reseau de stations</t>
@@ -1506,7 +1506,7 @@
       </c>
       <c r="D7" s="21" t="inlineStr">
         <is>
-          <t>cible — ultra-premium &amp; mobiles, prix ARSAT</t>
+          <t>cible — stations fixes et stations mobiles, prix ARSAT</t>
         </is>
       </c>
       <c r="E7" s="21" t="inlineStr">
@@ -1616,7 +1616,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="23.25" customHeight="1" s="15">
+    <row r="11" ht="34.5" customHeight="1" s="15">
       <c r="A11" s="21" t="inlineStr">
         <is>
           <t>Horizon long — transformation</t>
@@ -1624,7 +1624,7 @@
       </c>
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>250 kb/j · polymeres (PP, PE, PVC) · petrochimie avancee (olefines/aromatiques)</t>
+          <t>contribution à l'objectif national de 250 kb/j · polymeres (PP, PE, PVC) · petrochimie avancee (olefines/aromatiques)</t>
         </is>
       </c>
       <c r="C11" s="21" t="inlineStr">

</xml_diff>

<commit_message>
OVH: reviewed corporate readiness export from 85ff3ec9d945ecb9b775762ca28389d1838a0877
</commit_message>
<xml_diff>
--- a/Data_Book_EnerTchad.xlsx
+++ b/Data_Book_EnerTchad.xlsx
@@ -532,14 +532,14 @@
     <row r="11" ht="15" customHeight="1" s="15">
       <c r="A11" s="18" t="inlineStr">
         <is>
-          <t>Extraction : 18 octobre 2026, depuis le site officiel https://enertchad.com</t>
+          <t>Extraction : 18 octobre 2026, depuis le site officiel https://enertchad.com ; mise à jour : 23 octobre 2026</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="15">
       <c r="A12" s="18" t="inlineStr">
         <is>
-          <t>Contact investisseurs : contact@enertchad.com · +235 30 16 26 26 · Partenaire investissement : GCIC</t>
+          <t>Contact investisseurs : contact@enertchad.com · +235 30 16 26 26 · Conseil pressenti : GCIC</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="15">
+    <row r="9" ht="23.25" customHeight="1" s="15">
       <c r="A9" s="21" t="inlineStr">
         <is>
           <t>Organisation</t>
@@ -805,7 +805,7 @@
       </c>
       <c r="B9" s="21" t="inlineStr">
         <is>
-          <t>Societe unique (pas un groupe) — 3 poles de coeur, petrochimie, 4 capacites integrees</t>
+          <t>Société unique (pas un groupe) — 4 segments industriels + 4 capacités intégrées</t>
         </is>
       </c>
       <c r="C9" s="21" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="10" ht="15" customHeight="1" s="15">
       <c r="A10" s="20" t="inlineStr">
         <is>
-          <t>Poles chaine (4)</t>
+          <t>Segments industriels (4)</t>
         </is>
       </c>
       <c r="B10" s="20" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="11" ht="15" customHeight="1" s="15">
       <c r="A11" s="21" t="inlineStr">
         <is>
-          <t>Poles supports (4)</t>
+          <t>Capacités intégrées (4)</t>
         </is>
       </c>
       <c r="B11" s="21" t="inlineStr">
@@ -908,17 +908,17 @@
     <row r="13" ht="15" customHeight="1" s="15">
       <c r="A13" s="21" t="inlineStr">
         <is>
-          <t>Partenaire investissement</t>
+          <t>Conseil pressenti (levées)</t>
         </is>
       </c>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>GCIC</t>
+          <t>GCIC (Guess Consulting &amp; Investment Capital)</t>
         </is>
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
-          <t>fait</t>
+          <t>cible</t>
         </is>
       </c>
       <c r="D13" s="21" t="inlineStr">
@@ -1050,7 +1050,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="15">
+    <row r="4" ht="23.25" customHeight="1" s="15">
       <c r="A4" s="20" t="inlineStr">
         <is>
           <t>1re levee visee</t>
@@ -1068,7 +1068,7 @@
       </c>
       <c r="D4" s="20" t="inlineStr">
         <is>
-          <t>cible — court terme, tours d'amorcage avec GCIC ; montant non publie</t>
+          <t>cible — court terme, tours d'amorçage (GCIC, conseil pressenti) ; montant non publié</t>
         </is>
       </c>
       <c r="E4" s="20" t="inlineStr">
@@ -1114,10 +1114,10 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="15">
+    <row r="6" ht="23.25" customHeight="1" s="15">
       <c r="A6" s="20" t="inlineStr">
         <is>
-          <t>Capital vise a cinq ans</t>
+          <t>Capital visé</t>
         </is>
       </c>
       <c r="B6" s="20" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>cible — a cinq ans, levees successives ; montant non publie</t>
+          <t>cible — levées successives par paliers ; montant non publié</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
@@ -1210,10 +1210,10 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="15">
+    <row r="9" ht="23.25" customHeight="1" s="15">
       <c r="A9" s="21" t="inlineStr">
         <is>
-          <t>Data room &amp; rencontres (GCIC)</t>
+          <t>Data room &amp; rencontres (GCIC, conseil pressenti)</t>
         </is>
       </c>
       <c r="B9" s="21" t="inlineStr">
@@ -1328,10 +1328,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="15">
+    <row r="2" ht="23.25" customHeight="1" s="15">
       <c r="A2" s="20" t="inlineStr">
         <is>
-          <t>Production visee</t>
+          <t>Production nationale visée par le plan 2025-2030</t>
         </is>
       </c>
       <c r="B2" s="20" t="inlineStr">
@@ -1346,7 +1346,7 @@
       </c>
       <c r="D2" s="20" t="inlineStr">
         <is>
-          <t>cible 2030</t>
+          <t>contexte — EnerTchad y contribue ; pas une cible propre</t>
         </is>
       </c>
       <c r="E2" s="20" t="inlineStr">
@@ -1360,20 +1360,20 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" s="15">
+    <row r="3" ht="23.25" customHeight="1" s="15">
       <c r="A3" s="21" t="inlineStr">
         <is>
-          <t>Poles d'activite</t>
+          <t>Segments industriels + capacités intégrées</t>
         </is>
       </c>
       <c r="B3" s="21" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4 + 4</t>
         </is>
       </c>
       <c r="C3" s="21" t="inlineStr">
         <is>
-          <t>poles</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D3" s="21" t="inlineStr">
@@ -1424,7 +1424,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="15">
+    <row r="5" ht="23.25" customHeight="1" s="15">
       <c r="A5" s="21" t="inlineStr">
         <is>
           <t>Capital cible</t>
@@ -1442,7 +1442,7 @@
       </c>
       <c r="D5" s="21" t="inlineStr">
         <is>
-          <t>cible a cinq ans — levees successives, montant non publie</t>
+          <t>cible — levées successives par paliers, montant non publié</t>
         </is>
       </c>
       <c r="E5" s="21" t="inlineStr">
@@ -1452,7 +1452,7 @@
       </c>
       <c r="F5" s="21" t="inlineStr">
         <is>
-          <t>2031</t>
+          <t>par paliers</t>
         </is>
       </c>
     </row>
@@ -1488,7 +1488,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="15">
+    <row r="7" ht="23.25" customHeight="1" s="15">
       <c r="A7" s="21" t="inlineStr">
         <is>
           <t>Reseau de stations</t>
@@ -1506,7 +1506,7 @@
       </c>
       <c r="D7" s="21" t="inlineStr">
         <is>
-          <t>cible — ultra-premium &amp; mobiles, prix ARSAT</t>
+          <t>cible — stations fixes et stations mobiles, prix ARSAT</t>
         </is>
       </c>
       <c r="E7" s="21" t="inlineStr">
@@ -1616,7 +1616,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="23.25" customHeight="1" s="15">
+    <row r="11" ht="34.5" customHeight="1" s="15">
       <c r="A11" s="21" t="inlineStr">
         <is>
           <t>Horizon long — transformation</t>
@@ -1624,7 +1624,7 @@
       </c>
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>250 kb/j · polymeres (PP, PE, PVC) · petrochimie avancee (olefines/aromatiques)</t>
+          <t>contribution à l'objectif national de 250 kb/j · polymeres (PP, PE, PVC) · petrochimie avancee (olefines/aromatiques)</t>
         </is>
       </c>
       <c r="C11" s="21" t="inlineStr">

</xml_diff>

<commit_message>
Lot 98 (8/9) : cohérence des chiffres — pages, flux et documents régénérés
Fiche investisseur et point d'étape régénérés (4 + 4, titulaires nommés, novembre 2026) ; Data Book : oléoduc ~53 % avec le calcul ITIE/COTCO, Brent sourcé STEO EIA ; Cibles 2030 FR/EN : emplois ITIE 2023 p. 252 et base EnerTchad ; Carnets FR/EN : bandeau 22 oct. 2026 · n° 33 ; CP-2026-007 : 32 carnets (flux FR/EN, page EN) ; GreenTech EN : TRIR ; cartes Publications et vignettes Investisseurs datées novembre 2026 ; tailles sur les pages de pôles EN.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01924b9tNJjnMM63pEUTgBf9
</commit_message>
<xml_diff>
--- a/Data_Book_EnerTchad.xlsx
+++ b/Data_Book_EnerTchad.xlsx
@@ -532,7 +532,7 @@
     <row r="11" ht="15" customHeight="1" s="15">
       <c r="A11" s="18" t="inlineStr">
         <is>
-          <t>Extraction : 18 octobre 2026, depuis le site officiel https://enertchad.com ; mise à jour : 23 octobre 2026</t>
+          <t>Extraction : 18 octobre 2026, depuis le site officiel https://enertchad.com ; mise à jour : 1er novembre 2026 (lot 98)</t>
         </is>
       </c>
     </row>
@@ -1983,7 +1983,7 @@
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>consensus ~58 $ (fevrier) · ~85 $ (ete)</t>
+          <t>~58 $ (prévision EIA, février) · ~85 $ (moyenne de juin)</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
@@ -1993,12 +1993,12 @@
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>contexte — estimation a confirmer — source en cours de verification</t>
+          <t>contexte — STEO de l’EIA de février 2026 (feb26.pdf) et de juillet 2026 (jul26.pdf) ; repris de https://enertchad.com/investisseurs#marche</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>source a confirmer</t>
+          <t>https://www.eia.gov/outlooks/steo/archives/feb26.pdf · https://www.eia.gov/outlooks/steo/archives/jul26.pdf</t>
         </is>
       </c>
       <c r="F6" s="20" t="inlineStr">
@@ -2015,7 +2015,7 @@
       </c>
       <c r="B7" s="21" t="inlineStr">
         <is>
-          <t>~69</t>
+          <t>~69 $ (août) · ~84 $ (octobre)</t>
         </is>
       </c>
       <c r="C7" s="21" t="inlineStr">
@@ -2025,12 +2025,12 @@
       </c>
       <c r="D7" s="21" t="inlineStr">
         <is>
-          <t>contexte — estimation a confirmer — source en cours de verification</t>
+          <t>contexte — prévisions STEO de l’EIA d’août 2026 (aug26.pdf) et d’octobre 2026 (oct26.pdf) ; repris de https://enertchad.com/investisseurs#marche</t>
         </is>
       </c>
       <c r="E7" s="21" t="inlineStr">
         <is>
-          <t>source a confirmer</t>
+          <t>https://www.eia.gov/outlooks/steo/archives/aug26.pdf · https://www.eia.gov/outlooks/steo/archives/oct26.pdf</t>
         </is>
       </c>
       <c r="F7" s="21" t="inlineStr">
@@ -2111,7 +2111,7 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>~55</t>
+          <t>~53</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
@@ -2121,12 +2121,12 @@
       </c>
       <c r="D10" s="20" t="inlineStr">
         <is>
-          <t>contexte — ~45 % de capacité disponible (ITIE 2023, COTCO)</t>
+          <t>contexte — 48,15 Mb exportés en 2023 (ITIE 2023, p. 20), soit ~132 kb/j, pour 250 kb/j de capacité (COTCO) ; ~47 % disponibles</t>
         </is>
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>https://enertchad.com/investisseurs#marche</t>
+          <t>https://www.itie-tchad.com/wp-content/uploads/2026/07/Rapport-ITIE-Tchad-2023-version-finale-301225.pdf · https://cotco-sa.cm/en/cameroon-transportation-system/</t>
         </is>
       </c>
       <c r="F10" s="20" t="inlineStr">

</xml_diff>

<commit_message>
OVH: reviewed corporate readiness export from 4c9e817596be9c3f53d7c8cab661d029fc8ca3ae
</commit_message>
<xml_diff>
--- a/Data_Book_EnerTchad.xlsx
+++ b/Data_Book_EnerTchad.xlsx
@@ -532,7 +532,7 @@
     <row r="11" ht="15" customHeight="1" s="15">
       <c r="A11" s="18" t="inlineStr">
         <is>
-          <t>Extraction : 18 octobre 2026, depuis le site officiel https://enertchad.com ; mise à jour : 23 octobre 2026</t>
+          <t>Extraction : 18 octobre 2026, depuis le site officiel https://enertchad.com ; mise à jour : 1er novembre 2026 (lot 98)</t>
         </is>
       </c>
     </row>
@@ -1983,7 +1983,7 @@
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>consensus ~58 $ (fevrier) · ~85 $ (ete)</t>
+          <t>~58 $ (prévision EIA, février) · ~85 $ (moyenne de juin)</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
@@ -1993,12 +1993,12 @@
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>contexte — estimation a confirmer — source en cours de verification</t>
+          <t>contexte — STEO de l’EIA de février 2026 (feb26.pdf) et de juillet 2026 (jul26.pdf) ; repris de https://enertchad.com/investisseurs#marche</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>source a confirmer</t>
+          <t>https://www.eia.gov/outlooks/steo/archives/feb26.pdf · https://www.eia.gov/outlooks/steo/archives/jul26.pdf</t>
         </is>
       </c>
       <c r="F6" s="20" t="inlineStr">
@@ -2015,7 +2015,7 @@
       </c>
       <c r="B7" s="21" t="inlineStr">
         <is>
-          <t>~69</t>
+          <t>~69 $ (août) · ~84 $ (octobre)</t>
         </is>
       </c>
       <c r="C7" s="21" t="inlineStr">
@@ -2025,12 +2025,12 @@
       </c>
       <c r="D7" s="21" t="inlineStr">
         <is>
-          <t>contexte — estimation a confirmer — source en cours de verification</t>
+          <t>contexte — prévisions STEO de l’EIA d’août 2026 (aug26.pdf) et d’octobre 2026 (oct26.pdf) ; repris de https://enertchad.com/investisseurs#marche</t>
         </is>
       </c>
       <c r="E7" s="21" t="inlineStr">
         <is>
-          <t>source a confirmer</t>
+          <t>https://www.eia.gov/outlooks/steo/archives/aug26.pdf · https://www.eia.gov/outlooks/steo/archives/oct26.pdf</t>
         </is>
       </c>
       <c r="F7" s="21" t="inlineStr">
@@ -2111,7 +2111,7 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>~55</t>
+          <t>~53</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
@@ -2121,12 +2121,12 @@
       </c>
       <c r="D10" s="20" t="inlineStr">
         <is>
-          <t>contexte — ~45 % de capacité disponible (ITIE 2023, COTCO)</t>
+          <t>contexte — 48,15 Mb exportés en 2023 (ITIE 2023, p. 20), soit ~132 kb/j, pour 250 kb/j de capacité (COTCO) ; ~47 % disponibles</t>
         </is>
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>https://enertchad.com/investisseurs#marche</t>
+          <t>https://www.itie-tchad.com/wp-content/uploads/2026/07/Rapport-ITIE-Tchad-2023-version-finale-301225.pdf · https://cotco-sa.cm/en/cameroon-transportation-system/</t>
         </is>
       </c>
       <c r="F10" s="20" t="inlineStr">

</xml_diff>